<commit_message>
Re-render after hERG/interim note fix
</commit_message>
<xml_diff>
--- a/output/archive/MerrivossData/Client_Work/BP16/MV-2026-278/MV-2026-278_AssayWorksheet_092426_v03.xlsx
+++ b/output/archive/MerrivossData/Client_Work/BP16/MV-2026-278/MV-2026-278_AssayWorksheet_092426_v03.xlsx
@@ -992,7 +992,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>INTERIM: 11 of 18 results reported; remaining in progress</t>
+          <t>INTERIM: 11 of 18 planned rows reported; remaining in progress</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>INTERIM: 10 of 18 results reported; remaining in progress</t>
+          <t>INTERIM: 10 of 18 planned rows reported; remaining in progress</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage 8 review fixes: C-022
</commit_message>
<xml_diff>
--- a/output/archive/MerrivossData/Client_Work/BP16/MV-2026-278/MV-2026-278_AssayWorksheet_092426_v03.xlsx
+++ b/output/archive/MerrivossData/Client_Work/BP16/MV-2026-278/MV-2026-278_AssayWorksheet_092426_v03.xlsx
@@ -164,7 +164,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Control values for each isoform still need comparing with the historical range before release</t>
+        <t>Document the control comparison with historical records before final release.</t>
       </text>
     </comment>
   </commentList>
@@ -179,7 +179,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Hold the two most potent rows until the relabelled vial is confirmed. Do not quote them in the interim readout.</t>
+        <t>Keep final interpretation pending until the client confirms the relabelled vial against the accession record; do not assign the identity hold to particular result rows without that record.</t>
       </text>
     </comment>
   </commentList>
@@ -192,9 +192,9 @@
     <author>Helen Marchwood</author>
   </authors>
   <commentList>
-    <comment ref="D4" authorId="0" shapeId="0">
+    <comment ref="C3" authorId="0" shapeId="0">
       <text>
-        <t>Pending until the relabelled vial is matched against the sample log</t>
+        <t>Leave identity sign-off blank until the client confirmation is matched to the accession record.</t>
       </text>
     </comment>
   </commentList>
@@ -532,7 +532,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MV-2026-278 assay worksheet, interim</t>
+          <t>Merrivoss Bioanalysis Inc, a Tarnovell company | MV-2026-278 assay worksheet, interim</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Compounds tested</t>
+          <t>Study test article count</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1028,7 +1028,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Values above 50 µM are reported as &gt;50. Compounds below 1 µM: 4; below 10 µM: 5.</t>
+          <t>Human liver microsomes, midazolam 1'-hydroxylation. Values above 50 µM are reported as &gt;50. This is a partial result table; whole-set potency counts and final interpretation remain pending identity confirmation.</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1259,22 +1259,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Vial</t>
+          <t>Source record</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Compound</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Received</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Identity check</t>
+          <t>Client confirmation</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1291,142 +1291,62 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>V-0412</t>
+          <t>Study accession M26/BIO/06402</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>BP16-05482</t>
+          <t>Relabelled vial identity</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Javier Quintana</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>09/22/2026</t>
-        </is>
-      </c>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>V-0413</t>
+          <t>Accession receipt record</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>BP16-05472</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Javier Quintana</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>09/22/2026</t>
-        </is>
-      </c>
+          <t>Match vial label to client identity confirmation</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>V-0419 (relabelled)</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>To be confirmed</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>09/14/2026</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>V-0420</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>BP16-05400</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>V-0421</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>BP16-05422</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>